<commit_message>
Add week of 25 May menu and Jun 1-5 draft
- Week of 25 May 2026 menu file with associated new recipes
- Jun 1-5 tentative menu parked in menu-ideas.md with 7 new recipe files
  (claypot tofu, dry laksa, miso glazed eggplant, mushroom soup,
  prawn noodle soup, teriyaki chicken, Thai green curry)
- Updated dish rotation tracker and kitchen inventory

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -940,101 +940,269 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
+      <c r="A23" s="2" t="n">
+        <v>46167</v>
+      </c>
       <c r="B23" s="3">
         <f>IF(A23="","",TEXT(A23,"ddd"))</f>
         <v/>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Nasi lemak</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
+      <c r="A24" s="2" t="n">
+        <v>46167</v>
+      </c>
       <c r="B24" s="3">
         <f>IF(A24="","",TEXT(A24,"ddd"))</f>
         <v/>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Korean fried chicken wings</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026) — honey soy</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
+      <c r="A25" s="2" t="n">
+        <v>46167</v>
+      </c>
       <c r="B25" s="3">
         <f>IF(A25="","",TEXT(A25,"ddd"))</f>
         <v/>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Egg omelette</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
+      <c r="A26" s="2" t="n">
+        <v>46167</v>
+      </c>
       <c r="B26" s="3">
         <f>IF(A26="","",TEXT(A26,"ddd"))</f>
         <v/>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sambal kangkong</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
+      <c r="A27" s="2" t="n">
+        <v>46167</v>
+      </c>
       <c r="B27" s="3">
         <f>IF(A27="","",TEXT(A27,"ddd"))</f>
         <v/>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Ikan bilis</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
+      <c r="A28" s="2" t="n">
+        <v>46168</v>
+      </c>
       <c r="B28" s="3">
         <f>IF(A28="","",TEXT(A28,"ddd"))</f>
         <v/>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Beancurd meat rolls</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
+      <c r="A29" s="2" t="n">
+        <v>46168</v>
+      </c>
       <c r="B29" s="3">
         <f>IF(A29="","",TEXT(A29,"ddd"))</f>
         <v/>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fried yellow croaker</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
+      <c r="A30" s="2" t="n">
+        <v>46168</v>
+      </c>
       <c r="B30" s="3">
         <f>IF(A30="","",TEXT(A30,"ddd"))</f>
         <v/>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lotus root pork rib soup</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
+      <c r="A31" s="2" t="n">
+        <v>46170</v>
+      </c>
       <c r="B31" s="3">
         <f>IF(A31="","",TEXT(A31,"ddd"))</f>
         <v/>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Steamed egg tofu with minced pork</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026) — with dried scallop</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
+      <c r="A32" s="2" t="n">
+        <v>46170</v>
+      </c>
       <c r="B32" s="3">
         <f>IF(A32="","",TEXT(A32,"ddd"))</f>
         <v/>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Pandan chicken</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
+      <c r="A33" s="2" t="n">
+        <v>46170</v>
+      </c>
       <c r="B33" s="3">
         <f>IF(A33="","",TEXT(A33,"ddd"))</f>
         <v/>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
+      <c r="A34" s="2" t="n">
+        <v>46171</v>
+      </c>
       <c r="B34" s="3">
         <f>IF(A34="","",TEXT(A34,"ddd"))</f>
         <v/>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Beef stew</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
+      <c r="A35" s="2" t="n">
+        <v>46171</v>
+      </c>
       <c r="B35" s="3">
         <f>IF(A35="","",TEXT(A35,"ddd"))</f>
         <v/>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Garlic bread</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
+      <c r="A36" s="2" t="n">
+        <v>46168</v>
+      </c>
       <c r="B36" s="3">
         <f>IF(A36="","",TEXT(A36,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Japanese mushroom rice</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>planned (week of 25 May 2026)</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -2902,7 +3070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5200,6 +5368,261 @@
         <v/>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Korean fried chicken wings</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>21</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>3 sauces: honey soy / black pepper / spicy sweet</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Sambal kangkong</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Beancurd meat rolls</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>28</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Dim sum, prawn + pork filling</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Fried yellow croaker</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Fish</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Lotus root pork rib soup</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Steamed egg tofu with minced pork</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Egg</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>21</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>With dried scallop</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Pandan chicken</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>28</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Thai style</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Beef stew</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>35</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Roland's classic Western braise</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Garlic bread</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Egg omelette</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Egg</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Ikan bilis</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>14</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>For nasi lemak</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>7</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Generic placeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Fried yam shrimp</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Prawn</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>35</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Dim sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Japanese mushroom rice</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>28</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Takikomi gohan with shimeji/king oyster/shiitake</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H71"/>

</xml_diff>

<commit_message>
Lock in week of 1 Jun 2026 menu and add pregnancy-vet workflow
- Week file: Sun spinach ban mian, Mon eat-out, Tue mushroom + fishball
  soup + sticky pork belly, Wed cheesy baked rice, Thu claypot tofu +
  Yang Zhou fried rice, Fri fried beehoon + Thai fishcakes
- 8 new recipe files for the week's dishes
- Pregnancy-vet skill (Western + TCM lenses) and report for this week
- Rotation tracker: cook log + 6 new master entries
- Inventory: 7 new specialty items flagged Out for the shopping list

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -1206,66 +1206,174 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
+      <c r="A37" s="2" t="n">
+        <v>46173</v>
+      </c>
       <c r="B37" s="3">
         <f>IF(A37="","",TEXT(A37,"ddd"))</f>
         <v/>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Spinach ban mian</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
+      <c r="A38" s="2" t="n">
+        <v>46175</v>
+      </c>
       <c r="B38" s="3">
         <f>IF(A38="","",TEXT(A38,"ddd"))</f>
         <v/>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Japanese miso butter mushroom</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
+      <c r="A39" s="2" t="n">
+        <v>46175</v>
+      </c>
       <c r="B39" s="3">
         <f>IF(A39="","",TEXT(A39,"ddd"))</f>
         <v/>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Fishball minced pork soup</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
+      <c r="A40" s="2" t="n">
+        <v>46175</v>
+      </c>
       <c r="B40" s="3">
         <f>IF(A40="","",TEXT(A40,"ddd"))</f>
         <v/>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sticky pork belly</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
+      <c r="A41" s="2" t="n">
+        <v>46176</v>
+      </c>
       <c r="B41" s="3">
         <f>IF(A41="","",TEXT(A41,"ddd"))</f>
         <v/>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Cheesy baked rice</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
+      <c r="A42" s="2" t="n">
+        <v>46177</v>
+      </c>
       <c r="B42" s="3">
         <f>IF(A42="","",TEXT(A42,"ddd"))</f>
         <v/>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Claypot tofu</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
+      <c r="A43" s="2" t="n">
+        <v>46177</v>
+      </c>
       <c r="B43" s="3">
         <f>IF(A43="","",TEXT(A43,"ddd"))</f>
         <v/>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Yang Zhou fried rice</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
+      <c r="A44" s="2" t="n">
+        <v>46178</v>
+      </c>
       <c r="B44" s="3">
         <f>IF(A44="","",TEXT(A44,"ddd"))</f>
         <v/>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Stir fried bee hoon</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
+      <c r="A45" s="2" t="n">
+        <v>46178</v>
+      </c>
       <c r="B45" s="3">
         <f>IF(A45="","",TEXT(A45,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Thai fishcakes</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>planned (week of 1 Jun 2026)</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -3070,7 +3178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5621,6 +5729,218 @@
       <c r="H85" t="inlineStr">
         <is>
           <t>Takikomi gohan with shimeji/king oyster/shiitake</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Spinach ban mian</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C86">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A86)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A86)),"")</f>
+        <v/>
+      </c>
+      <c r="D86">
+        <f>IF(C86="","",TODAY()-C86)</f>
+        <v/>
+      </c>
+      <c r="E86">
+        <f>COUNTIF('Cook log'!C2:C1000,A86)</f>
+        <v/>
+      </c>
+      <c r="F86" t="n">
+        <v>21</v>
+      </c>
+      <c r="G86">
+        <f>IF(C86="","Never cooked",IF(D86&lt;F86,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+      <c r="H86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Japanese miso butter mushroom</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C87">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A87)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A87)),"")</f>
+        <v/>
+      </c>
+      <c r="D87">
+        <f>IF(C87="","",TODAY()-C87)</f>
+        <v/>
+      </c>
+      <c r="E87">
+        <f>COUNTIF('Cook log'!C2:C1000,A87)</f>
+        <v/>
+      </c>
+      <c r="F87" t="n">
+        <v>28</v>
+      </c>
+      <c r="G87">
+        <f>IF(C87="","Never cooked",IF(D87&lt;F87,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Foil yaki, assorted Japanese mushrooms</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Fishball minced pork soup</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C88">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A88)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A88)),"")</f>
+        <v/>
+      </c>
+      <c r="D88">
+        <f>IF(C88="","",TODAY()-C88)</f>
+        <v/>
+      </c>
+      <c r="E88">
+        <f>COUNTIF('Cook log'!C2:C1000,A88)</f>
+        <v/>
+      </c>
+      <c r="F88" t="n">
+        <v>21</v>
+      </c>
+      <c r="G88">
+        <f>IF(C88="","Never cooked",IF(D88&lt;F88,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Adaptable — add blanched leafy greens</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Cheesy baked rice</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C89">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A89)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A89)),"")</f>
+        <v/>
+      </c>
+      <c r="D89">
+        <f>IF(C89="","",TODAY()-C89)</f>
+        <v/>
+      </c>
+      <c r="E89">
+        <f>COUNTIF('Cook log'!C2:C1000,A89)</f>
+        <v/>
+      </c>
+      <c r="F89" t="n">
+        <v>28</v>
+      </c>
+      <c r="G89">
+        <f>IF(C89="","Never cooked",IF(D89&lt;F89,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Family recipe (Pa) — seafood + cheese</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Claypot tofu</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Egg</t>
+        </is>
+      </c>
+      <c r="C90">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A90)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A90)),"")</f>
+        <v/>
+      </c>
+      <c r="D90">
+        <f>IF(C90="","",TODAY()-C90)</f>
+        <v/>
+      </c>
+      <c r="E90">
+        <f>COUNTIF('Cook log'!C2:C1000,A90)</f>
+        <v/>
+      </c>
+      <c r="F90" t="n">
+        <v>21</v>
+      </c>
+      <c r="G90">
+        <f>IF(C90="","Never cooked",IF(D90&lt;F90,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Egg tofu, doubanjiang, minced pork, prawns</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Yang Zhou fried rice</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C91">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A91)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A91)),"")</f>
+        <v/>
+      </c>
+      <c r="D91">
+        <f>IF(C91="","",TODAY()-C91)</f>
+        <v/>
+      </c>
+      <c r="E91">
+        <f>COUNTIF('Cook log'!C2:C1000,A91)</f>
+        <v/>
+      </c>
+      <c r="F91" t="n">
+        <v>28</v>
+      </c>
+      <c r="G91">
+        <f>IF(C91="","Never cooked",IF(D91&lt;F91,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>With jin hua ham</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add weeks of 8 Jun & 15 Jun menus, vets, and recipe library
- Lock in week of 8 Jun 2026 menu + T1 pregnancy vet
- Lock in week of 15 Jun 2026 menu + T1 pregnancy vet
- Add ~35 new recipe files (noodles, rice, soups, seafood, veg, etc.)
- Update dish-rotation cook log + master for both weeks
- Update kitchen-inventory with new specialty items (Out)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -1377,157 +1377,421 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
+      <c r="A46" s="2" t="n">
+        <v>46181</v>
+      </c>
       <c r="B46" s="3">
         <f>IF(A46="","",TEXT(A46,"ddd"))</f>
         <v/>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Prawn noodle soup</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
+      <c r="A47" s="2" t="n">
+        <v>46182</v>
+      </c>
       <c r="B47" s="3">
         <f>IF(A47="","",TEXT(A47,"ddd"))</f>
         <v/>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Steamed pomfret</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
+      <c r="A48" s="2" t="n">
+        <v>46182</v>
+      </c>
       <c r="B48" s="3">
         <f>IF(A48="","",TEXT(A48,"ddd"))</f>
         <v/>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Stir fried dou miao</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
+      <c r="A49" s="2" t="n">
+        <v>46182</v>
+      </c>
       <c r="B49" s="3">
         <f>IF(A49="","",TEXT(A49,"ddd"))</f>
         <v/>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Tomato egg</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n"/>
+      <c r="A50" s="2" t="n">
+        <v>46183</v>
+      </c>
       <c r="B50" s="3">
         <f>IF(A50="","",TEXT(A50,"ddd"))</f>
         <v/>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Baked salmon with herbs</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
+      <c r="A51" s="2" t="n">
+        <v>46183</v>
+      </c>
       <c r="B51" s="3">
         <f>IF(A51="","",TEXT(A51,"ddd"))</f>
         <v/>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Roasted vegetables (oven)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026) — grilled veg</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
+      <c r="A52" s="2" t="n">
+        <v>46183</v>
+      </c>
       <c r="B52" s="3">
         <f>IF(A52="","",TEXT(A52,"ddd"))</f>
         <v/>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Mushroom soup</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
+      <c r="A53" s="2" t="n">
+        <v>46183</v>
+      </c>
       <c r="B53" s="3">
         <f>IF(A53="","",TEXT(A53,"ddd"))</f>
         <v/>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Garlic bread</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
+      <c r="A54" s="2" t="n">
+        <v>46184</v>
+      </c>
       <c r="B54" s="3">
         <f>IF(A54="","",TEXT(A54,"ddd"))</f>
         <v/>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Stir-fry beef ramen</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
+      <c r="A55" s="2" t="n">
+        <v>46184</v>
+      </c>
       <c r="B55" s="3">
         <f>IF(A55="","",TEXT(A55,"ddd"))</f>
         <v/>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Radish pork rib soup with dates</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
+      <c r="A56" s="2" t="n">
+        <v>46185</v>
+      </c>
       <c r="B56" s="3">
         <f>IF(A56="","",TEXT(A56,"ddd"))</f>
         <v/>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>HK steamed chicken rice</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>planned (week of 8 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n"/>
+      <c r="A57" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="B57" s="3">
         <f>IF(A57="","",TEXT(A57,"ddd"))</f>
         <v/>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Claypot Mee Tai Bak</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
+      <c r="A58" s="2" t="n">
+        <v>46189</v>
+      </c>
       <c r="B58" s="3">
         <f>IF(A58="","",TEXT(A58,"ddd"))</f>
         <v/>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Fried threadfin with onion</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
+      <c r="A59" s="2" t="n">
+        <v>46189</v>
+      </c>
       <c r="B59" s="3">
         <f>IF(A59="","",TEXT(A59,"ddd"))</f>
         <v/>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Stir-fried eggs and prawns</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
+      <c r="A60" s="2" t="n">
+        <v>46189</v>
+      </c>
       <c r="B60" s="3">
         <f>IF(A60="","",TEXT(A60,"ddd"))</f>
         <v/>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Hainanese chap chye</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
+      <c r="A61" s="2" t="n">
+        <v>46190</v>
+      </c>
       <c r="B61" s="3">
         <f>IF(A61="","",TEXT(A61,"ddd"))</f>
         <v/>
       </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Shimeji spinach tofu</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
+      <c r="A62" s="2" t="n">
+        <v>46191</v>
+      </c>
       <c r="B62" s="3">
         <f>IF(A62="","",TEXT(A62,"ddd"))</f>
         <v/>
       </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Taiwanese fried rice</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
+      <c r="A63" s="2" t="n">
+        <v>46191</v>
+      </c>
       <c r="B63" s="3">
         <f>IF(A63="","",TEXT(A63,"ddd"))</f>
         <v/>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Tonjiru</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
+      <c r="A64" s="2" t="n">
+        <v>46192</v>
+      </c>
       <c r="B64" s="3">
         <f>IF(A64="","",TEXT(A64,"ddd"))</f>
         <v/>
       </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chicken chop &amp; mushroom noodles</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
+      <c r="A65" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="B65" s="3">
         <f>IF(A65="","",TEXT(A65,"ddd"))</f>
         <v/>
       </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Watercress pork rib soup</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n"/>
+      <c r="A66" s="2" t="n">
+        <v>46190</v>
+      </c>
       <c r="B66" s="3">
         <f>IF(A66="","",TEXT(A66,"ddd"))</f>
         <v/>
       </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Stir-fried eggplant and long bean with dried shrimp</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n"/>
+      <c r="A67" s="2" t="n">
+        <v>46190</v>
+      </c>
       <c r="B67" s="3">
         <f>IF(A67="","",TEXT(A67,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Spring onion beef stir fry</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>planned (week of 15 Jun 2026)</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -3178,7 +3442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5762,7 +6026,6 @@
         <f>IF(C86="","Never cooked",IF(D86&lt;F86,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5942,6 +6205,533 @@
         <is>
           <t>With jin hua ham</t>
         </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Prawn noodle soup</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C92">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A92)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A92)),"")</f>
+        <v/>
+      </c>
+      <c r="D92">
+        <f>IF(C92="","",TODAY()-C92)</f>
+        <v/>
+      </c>
+      <c r="E92">
+        <f>COUNTIF('Cook log'!C2:C1000,A92)</f>
+        <v/>
+      </c>
+      <c r="F92" t="n">
+        <v>21</v>
+      </c>
+      <c r="G92">
+        <f>IF(C92="","Never cooked",IF(D92&lt;F92,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Baked salmon with herbs</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Fish</t>
+        </is>
+      </c>
+      <c r="C93">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A93)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A93)),"")</f>
+        <v/>
+      </c>
+      <c r="D93">
+        <f>IF(C93="","",TODAY()-C93)</f>
+        <v/>
+      </c>
+      <c r="E93">
+        <f>COUNTIF('Cook log'!C2:C1000,A93)</f>
+        <v/>
+      </c>
+      <c r="F93" t="n">
+        <v>21</v>
+      </c>
+      <c r="G93">
+        <f>IF(C93="","Never cooked",IF(D93&lt;F93,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Stir-fry beef ramen</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C94">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A94)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A94)),"")</f>
+        <v/>
+      </c>
+      <c r="D94">
+        <f>IF(C94="","",TODAY()-C94)</f>
+        <v/>
+      </c>
+      <c r="E94">
+        <f>COUNTIF('Cook log'!C2:C1000,A94)</f>
+        <v/>
+      </c>
+      <c r="F94" t="n">
+        <v>21</v>
+      </c>
+      <c r="G94">
+        <f>IF(C94="","Never cooked",IF(D94&lt;F94,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>HK steamed chicken rice</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C95">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A95)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A95)),"")</f>
+        <v/>
+      </c>
+      <c r="D95">
+        <f>IF(C95="","",TODAY()-C95)</f>
+        <v/>
+      </c>
+      <c r="E95">
+        <f>COUNTIF('Cook log'!C2:C1000,A95)</f>
+        <v/>
+      </c>
+      <c r="F95" t="n">
+        <v>21</v>
+      </c>
+      <c r="G95">
+        <f>IF(C95="","Never cooked",IF(D95&lt;F95,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Wat Tan Hor Fun</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C96">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A96)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A96)),"")</f>
+        <v/>
+      </c>
+      <c r="D96">
+        <f>IF(C96="","",TODAY()-C96)</f>
+        <v/>
+      </c>
+      <c r="E96">
+        <f>COUNTIF('Cook log'!C2:C1000,A96)</f>
+        <v/>
+      </c>
+      <c r="F96" t="n">
+        <v>21</v>
+      </c>
+      <c r="G96">
+        <f>IF(C96="","Never cooked",IF(D96&lt;F96,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Seafood pao fan</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C97">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A97)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A97)),"")</f>
+        <v/>
+      </c>
+      <c r="D97">
+        <f>IF(C97="","",TODAY()-C97)</f>
+        <v/>
+      </c>
+      <c r="E97">
+        <f>COUNTIF('Cook log'!C2:C1000,A97)</f>
+        <v/>
+      </c>
+      <c r="F97" t="n">
+        <v>21</v>
+      </c>
+      <c r="G97">
+        <f>IF(C97="","Never cooked",IF(D97&lt;F97,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Pepper lunch beef rice</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C98">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A98)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A98)),"")</f>
+        <v/>
+      </c>
+      <c r="D98">
+        <f>IF(C98="","",TODAY()-C98)</f>
+        <v/>
+      </c>
+      <c r="E98">
+        <f>COUNTIF('Cook log'!C2:C1000,A98)</f>
+        <v/>
+      </c>
+      <c r="F98" t="n">
+        <v>21</v>
+      </c>
+      <c r="G98">
+        <f>IF(C98="","Never cooked",IF(D98&lt;F98,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Tonjiru</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C99">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A99)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A99)),"")</f>
+        <v/>
+      </c>
+      <c r="D99">
+        <f>IF(C99="","",TODAY()-C99)</f>
+        <v/>
+      </c>
+      <c r="E99">
+        <f>COUNTIF('Cook log'!C2:C1000,A99)</f>
+        <v/>
+      </c>
+      <c r="F99" t="n">
+        <v>21</v>
+      </c>
+      <c r="G99">
+        <f>IF(C99="","Never cooked",IF(D99&lt;F99,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Chicken chop &amp; mushroom noodles</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C100">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A100)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A100)),"")</f>
+        <v/>
+      </c>
+      <c r="D100">
+        <f>IF(C100="","",TODAY()-C100)</f>
+        <v/>
+      </c>
+      <c r="E100">
+        <f>COUNTIF('Cook log'!C2:C1000,A100)</f>
+        <v/>
+      </c>
+      <c r="F100" t="n">
+        <v>21</v>
+      </c>
+      <c r="G100">
+        <f>IF(C100="","Never cooked",IF(D100&lt;F100,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Stir-fried eggs and prawns</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Prawn</t>
+        </is>
+      </c>
+      <c r="C101">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A101)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A101)),"")</f>
+        <v/>
+      </c>
+      <c r="D101">
+        <f>IF(C101="","",TODAY()-C101)</f>
+        <v/>
+      </c>
+      <c r="E101">
+        <f>COUNTIF('Cook log'!C2:C1000,A101)</f>
+        <v/>
+      </c>
+      <c r="F101" t="n">
+        <v>21</v>
+      </c>
+      <c r="G101">
+        <f>IF(C101="","Never cooked",IF(D101&lt;F101,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Claypot Mee Tai Bak</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C102">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A102)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A102)),"")</f>
+        <v/>
+      </c>
+      <c r="D102">
+        <f>IF(C102="","",TODAY()-C102)</f>
+        <v/>
+      </c>
+      <c r="E102">
+        <f>COUNTIF('Cook log'!C2:C1000,A102)</f>
+        <v/>
+      </c>
+      <c r="F102" t="n">
+        <v>21</v>
+      </c>
+      <c r="G102">
+        <f>IF(C102="","Never cooked",IF(D102&lt;F102,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Fried threadfin with onion</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Fish</t>
+        </is>
+      </c>
+      <c r="C103">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A103)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A103)),"")</f>
+        <v/>
+      </c>
+      <c r="D103">
+        <f>IF(C103="","",TODAY()-C103)</f>
+        <v/>
+      </c>
+      <c r="E103">
+        <f>COUNTIF('Cook log'!C2:C1000,A103)</f>
+        <v/>
+      </c>
+      <c r="F103" t="n">
+        <v>21</v>
+      </c>
+      <c r="G103">
+        <f>IF(C103="","Never cooked",IF(D103&lt;F103,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Hainanese chap chye</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C104">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A104)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A104)),"")</f>
+        <v/>
+      </c>
+      <c r="D104">
+        <f>IF(C104="","",TODAY()-C104)</f>
+        <v/>
+      </c>
+      <c r="E104">
+        <f>COUNTIF('Cook log'!C2:C1000,A104)</f>
+        <v/>
+      </c>
+      <c r="F104" t="n">
+        <v>21</v>
+      </c>
+      <c r="G104">
+        <f>IF(C104="","Never cooked",IF(D104&lt;F104,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Shimeji spinach tofu</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C105">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A105)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A105)),"")</f>
+        <v/>
+      </c>
+      <c r="D105">
+        <f>IF(C105="","",TODAY()-C105)</f>
+        <v/>
+      </c>
+      <c r="E105">
+        <f>COUNTIF('Cook log'!C2:C1000,A105)</f>
+        <v/>
+      </c>
+      <c r="F105" t="n">
+        <v>21</v>
+      </c>
+      <c r="G105">
+        <f>IF(C105="","Never cooked",IF(D105&lt;F105,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Stir-fried eggplant and long bean with dried shrimp</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C106">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A106)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A106)),"")</f>
+        <v/>
+      </c>
+      <c r="D106">
+        <f>IF(C106="","",TODAY()-C106)</f>
+        <v/>
+      </c>
+      <c r="E106">
+        <f>COUNTIF('Cook log'!C2:C1000,A106)</f>
+        <v/>
+      </c>
+      <c r="F106" t="n">
+        <v>21</v>
+      </c>
+      <c r="G106">
+        <f>IF(C106="","Never cooked",IF(D106&lt;F106,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Spring onion beef stir fry</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="C107">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A107)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A107)),"")</f>
+        <v/>
+      </c>
+      <c r="D107">
+        <f>IF(C107="","",TODAY()-C107)</f>
+        <v/>
+      </c>
+      <c r="E107">
+        <f>COUNTIF('Cook log'!C2:C1000,A107)</f>
+        <v/>
+      </c>
+      <c r="F107" t="n">
+        <v>21</v>
+      </c>
+      <c r="G107">
+        <f>IF(C107="","Never cooked",IF(D107&lt;F107,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Taiwanese fried rice</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C108">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A108)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A108)),"")</f>
+        <v/>
+      </c>
+      <c r="D108">
+        <f>IF(C108="","",TODAY()-C108)</f>
+        <v/>
+      </c>
+      <c r="E108">
+        <f>COUNTIF('Cook log'!C2:C1000,A108)</f>
+        <v/>
+      </c>
+      <c r="F108" t="n">
+        <v>21</v>
+      </c>
+      <c r="G108">
+        <f>IF(C108="","Never cooked",IF(D108&lt;F108,"Cooldown","Due"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add week of 22 Jun 2026 menu, vet, and 9 new recipes
- Lock in week of 22 Jun 2026 menu (tomato + Korean themed) + T1 vet
- Add recipes: bolognese, spicy gochujang noodles, HK baked pork chop rice,
  Chinese yam & chicken soup, minestrone, steamed stuffed tofu puffs,
  potato/carrot minced pork, ngoh hiang, sweet & sour prawns on silky eggs
- Update dish-rotation cook log + master for the week
- Update kitchen-inventory with new specialty items (Out)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -1795,94 +1795,250 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n"/>
+      <c r="A68" s="2" t="n">
+        <v>46194</v>
+      </c>
       <c r="B68" s="3">
         <f>IF(A68="","",TEXT(A68,"ddd"))</f>
         <v/>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Minestrone soup</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
+      <c r="A69" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="B69" s="3">
         <f>IF(A69="","",TEXT(A69,"ddd"))</f>
         <v/>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Chinese yam and chicken soup</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n"/>
+      <c r="A70" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="B70" s="3">
         <f>IF(A70="","",TEXT(A70,"ddd"))</f>
         <v/>
       </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Pork rib king</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n"/>
+      <c r="A71" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="B71" s="3">
         <f>IF(A71="","",TEXT(A71,"ddd"))</f>
         <v/>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
+      <c r="A72" s="2" t="n">
+        <v>46196</v>
+      </c>
       <c r="B72" s="3">
         <f>IF(A72="","",TEXT(A72,"ddd"))</f>
         <v/>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Korean fried chicken wings</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026) — soy</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n"/>
+      <c r="A73" s="2" t="n">
+        <v>46196</v>
+      </c>
       <c r="B73" s="3">
         <f>IF(A73="","",TEXT(A73,"ddd"))</f>
         <v/>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Tomato egg</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n"/>
+      <c r="A74" s="2" t="n">
+        <v>46196</v>
+      </c>
       <c r="B74" s="3">
         <f>IF(A74="","",TEXT(A74,"ddd"))</f>
         <v/>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Lotus root pork rib soup</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n"/>
+      <c r="A75" s="2" t="n">
+        <v>46197</v>
+      </c>
       <c r="B75" s="3">
         <f>IF(A75="","",TEXT(A75,"ddd"))</f>
         <v/>
       </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Stir fried bee hoon</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026) — Sin Chew style</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n"/>
+      <c r="A76" s="2" t="n">
+        <v>46197</v>
+      </c>
       <c r="B76" s="3">
         <f>IF(A76="","",TEXT(A76,"ddd"))</f>
         <v/>
       </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Fishball and baby spinach soup</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n"/>
+      <c r="A77" s="2" t="n">
+        <v>46198</v>
+      </c>
       <c r="B77" s="3">
         <f>IF(A77="","",TEXT(A77,"ddd"))</f>
         <v/>
       </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Stir-fried potatoes &amp; carrots with minced meat</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026) — + tomato</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n"/>
+      <c r="A78" s="2" t="n">
+        <v>46198</v>
+      </c>
       <c r="B78" s="3">
         <f>IF(A78="","",TEXT(A78,"ddd"))</f>
         <v/>
       </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Fried fish with Thai sweet chilli</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n"/>
+      <c r="A79" s="2" t="n">
+        <v>46198</v>
+      </c>
       <c r="B79" s="3">
         <f>IF(A79="","",TEXT(A79,"ddd"))</f>
         <v/>
       </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Steamed egg (ah gong style)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n"/>
+      <c r="A80" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="B80" s="3">
         <f>IF(A80="","",TEXT(A80,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>HK baked pork chop rice</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>planned (week of 22 Jun 2026)</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -3442,7 +3598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6731,6 +6887,285 @@
       </c>
       <c r="G108">
         <f>IF(C108="","Never cooked",IF(D108&lt;F108,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Bolognese</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C109">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A109)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A109)),"")</f>
+        <v/>
+      </c>
+      <c r="D109">
+        <f>IF(C109="","",TODAY()-C109)</f>
+        <v/>
+      </c>
+      <c r="E109">
+        <f>COUNTIF('Cook log'!C2:C1000,A109)</f>
+        <v/>
+      </c>
+      <c r="F109" t="n">
+        <v>21</v>
+      </c>
+      <c r="G109">
+        <f>IF(C109="","Never cooked",IF(D109&lt;F109,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Spicy gochujang noodles</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C110">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A110)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A110)),"")</f>
+        <v/>
+      </c>
+      <c r="D110">
+        <f>IF(C110="","",TODAY()-C110)</f>
+        <v/>
+      </c>
+      <c r="E110">
+        <f>COUNTIF('Cook log'!C2:C1000,A110)</f>
+        <v/>
+      </c>
+      <c r="F110" t="n">
+        <v>21</v>
+      </c>
+      <c r="G110">
+        <f>IF(C110="","Never cooked",IF(D110&lt;F110,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Miso glazed eggplant</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C111">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A111)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A111)),"")</f>
+        <v/>
+      </c>
+      <c r="D111">
+        <f>IF(C111="","",TODAY()-C111)</f>
+        <v/>
+      </c>
+      <c r="E111">
+        <f>COUNTIF('Cook log'!C2:C1000,A111)</f>
+        <v/>
+      </c>
+      <c r="F111" t="n">
+        <v>21</v>
+      </c>
+      <c r="G111">
+        <f>IF(C111="","Never cooked",IF(D111&lt;F111,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Minestrone soup</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C112">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A112)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A112)),"")</f>
+        <v/>
+      </c>
+      <c r="D112">
+        <f>IF(C112="","",TODAY()-C112)</f>
+        <v/>
+      </c>
+      <c r="E112">
+        <f>COUNTIF('Cook log'!C2:C1000,A112)</f>
+        <v/>
+      </c>
+      <c r="F112" t="n">
+        <v>21</v>
+      </c>
+      <c r="G112">
+        <f>IF(C112="","Never cooked",IF(D112&lt;F112,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Chinese yam and chicken soup</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C113">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A113)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A113)),"")</f>
+        <v/>
+      </c>
+      <c r="D113">
+        <f>IF(C113="","",TODAY()-C113)</f>
+        <v/>
+      </c>
+      <c r="E113">
+        <f>COUNTIF('Cook log'!C2:C1000,A113)</f>
+        <v/>
+      </c>
+      <c r="F113" t="n">
+        <v>21</v>
+      </c>
+      <c r="G113">
+        <f>IF(C113="","Never cooked",IF(D113&lt;F113,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Fishball and baby spinach soup</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C114">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A114)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A114)),"")</f>
+        <v/>
+      </c>
+      <c r="D114">
+        <f>IF(C114="","",TODAY()-C114)</f>
+        <v/>
+      </c>
+      <c r="E114">
+        <f>COUNTIF('Cook log'!C2:C1000,A114)</f>
+        <v/>
+      </c>
+      <c r="F114" t="n">
+        <v>21</v>
+      </c>
+      <c r="G114">
+        <f>IF(C114="","Never cooked",IF(D114&lt;F114,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Stir-fried potatoes &amp; carrots with minced meat</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="C115">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A115)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A115)),"")</f>
+        <v/>
+      </c>
+      <c r="D115">
+        <f>IF(C115="","",TODAY()-C115)</f>
+        <v/>
+      </c>
+      <c r="E115">
+        <f>COUNTIF('Cook log'!C2:C1000,A115)</f>
+        <v/>
+      </c>
+      <c r="F115" t="n">
+        <v>21</v>
+      </c>
+      <c r="G115">
+        <f>IF(C115="","Never cooked",IF(D115&lt;F115,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Fried fish with Thai sweet chilli</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Fish</t>
+        </is>
+      </c>
+      <c r="C116">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A116)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A116)),"")</f>
+        <v/>
+      </c>
+      <c r="D116">
+        <f>IF(C116="","",TODAY()-C116)</f>
+        <v/>
+      </c>
+      <c r="E116">
+        <f>COUNTIF('Cook log'!C2:C1000,A116)</f>
+        <v/>
+      </c>
+      <c r="F116" t="n">
+        <v>21</v>
+      </c>
+      <c r="G116">
+        <f>IF(C116="","Never cooked",IF(D116&lt;F116,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>HK baked pork chop rice</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C117">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A117)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A117)),"")</f>
+        <v/>
+      </c>
+      <c r="D117">
+        <f>IF(C117="","",TODAY()-C117)</f>
+        <v/>
+      </c>
+      <c r="E117">
+        <f>COUNTIF('Cook log'!C2:C1000,A117)</f>
+        <v/>
+      </c>
+      <c r="F117" t="n">
+        <v>21</v>
+      </c>
+      <c r="G117">
+        <f>IF(C117="","Never cooked",IF(D117&lt;F117,"Cooldown","Due"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add week of 29 Jun 2026 (potato-themed) menu, vet, and recipes
- Lock in week of 29 Jun 2026 menu + T1 vet (potato dish every day;
  Sun shepherd's pie beef mince 2-pax; Wed Japanese curry cubes)
- Add 20 recipes: shepherd's pie, the potato collection (aligot, gratin,
  dauphinoise, roast, baked, croquettes, frittata, patatas bravas, begedil,
  parmesan wedges, nikujaga, leek soup, luncheon-meat x2), oven baked
  chicken leg, baked pork chops, teriyaki pork chop, thai steamed fish,
  kimchi pancake
- Update dish-rotation cook log + master for the week
- Update kitchen-inventory with new specialty items (Out)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -2042,108 +2042,288 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n"/>
+      <c r="A81" s="2" t="n">
+        <v>46201</v>
+      </c>
       <c r="B81" s="3">
         <f>IF(A81="","",TEXT(A81,"ddd"))</f>
         <v/>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Shepherd's pie</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026) — beef mince, 2 pax</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n"/>
+      <c r="A82" s="2" t="n">
+        <v>46202</v>
+      </c>
       <c r="B82" s="3">
         <f>IF(A82="","",TEXT(A82,"ddd"))</f>
         <v/>
       </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Potato gratin</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026) — au gratin</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n"/>
+      <c r="A83" s="2" t="n">
+        <v>46202</v>
+      </c>
       <c r="B83" s="3">
         <f>IF(A83="","",TEXT(A83,"ddd"))</f>
         <v/>
       </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Oven baked chicken leg</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n"/>
+      <c r="A84" s="2" t="n">
+        <v>46202</v>
+      </c>
       <c r="B84" s="3">
         <f>IF(A84="","",TEXT(A84,"ddd"))</f>
         <v/>
       </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Grilled asparagus</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n"/>
+      <c r="A85" s="2" t="n">
+        <v>46203</v>
+      </c>
       <c r="B85" s="3">
         <f>IF(A85="","",TEXT(A85,"ddd"))</f>
         <v/>
       </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Baked potatoes</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n"/>
+      <c r="A86" s="2" t="n">
+        <v>46203</v>
+      </c>
       <c r="B86" s="3">
         <f>IF(A86="","",TEXT(A86,"ddd"))</f>
         <v/>
       </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Chicken chop</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n"/>
+      <c r="A87" s="2" t="n">
+        <v>46203</v>
+      </c>
       <c r="B87" s="3">
         <f>IF(A87="","",TEXT(A87,"ddd"))</f>
         <v/>
       </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Roasted vegetables (oven)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n"/>
+      <c r="A88" s="2" t="n">
+        <v>46204</v>
+      </c>
       <c r="B88" s="3">
         <f>IF(A88="","",TEXT(A88,"ddd"))</f>
         <v/>
       </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Japanese curry rice</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026) — curry cubes</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n"/>
+      <c r="A89" s="2" t="n">
+        <v>46204</v>
+      </c>
       <c r="B89" s="3">
         <f>IF(A89="","",TEXT(A89,"ddd"))</f>
         <v/>
       </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Campbell's mushroom soup</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n"/>
+      <c r="A90" s="2" t="n">
+        <v>46205</v>
+      </c>
       <c r="B90" s="3">
         <f>IF(A90="","",TEXT(A90,"ddd"))</f>
         <v/>
       </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Radish pork rib soup with dates</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n"/>
+      <c r="A91" s="2" t="n">
+        <v>46205</v>
+      </c>
       <c r="B91" s="3">
         <f>IF(A91="","",TEXT(A91,"ddd"))</f>
         <v/>
       </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Stir-fried potatoes &amp; carrots with minced meat</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026) — + tomato</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n"/>
+      <c r="A92" s="2" t="n">
+        <v>46205</v>
+      </c>
       <c r="B92" s="3">
         <f>IF(A92="","",TEXT(A92,"ddd"))</f>
         <v/>
       </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Egg omelette</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026) — onion</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n"/>
+      <c r="A93" s="2" t="n">
+        <v>46206</v>
+      </c>
       <c r="B93" s="3">
         <f>IF(A93="","",TEXT(A93,"ddd"))</f>
         <v/>
       </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Crispy roast potatoes</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n"/>
+      <c r="A94" s="2" t="n">
+        <v>46206</v>
+      </c>
       <c r="B94" s="3">
         <f>IF(A94="","",TEXT(A94,"ddd"))</f>
         <v/>
       </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Baked pork chops</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n"/>
+      <c r="A95" s="2" t="n">
+        <v>46206</v>
+      </c>
       <c r="B95" s="3">
         <f>IF(A95="","",TEXT(A95,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Grilled broccoli &amp; carrots</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>planned (week of 29 Jun 2026)</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -3598,7 +3778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7166,6 +7346,347 @@
       </c>
       <c r="G117">
         <f>IF(C117="","Never cooked",IF(D117&lt;F117,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Shepherd's pie</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C118">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A118)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A118)),"")</f>
+        <v/>
+      </c>
+      <c r="D118">
+        <f>IF(C118="","",TODAY()-C118)</f>
+        <v/>
+      </c>
+      <c r="E118">
+        <f>COUNTIF('Cook log'!C2:C1000,A118)</f>
+        <v/>
+      </c>
+      <c r="F118" t="n">
+        <v>21</v>
+      </c>
+      <c r="G118">
+        <f>IF(C118="","Never cooked",IF(D118&lt;F118,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Potato gratin</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C119">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A119)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A119)),"")</f>
+        <v/>
+      </c>
+      <c r="D119">
+        <f>IF(C119="","",TODAY()-C119)</f>
+        <v/>
+      </c>
+      <c r="E119">
+        <f>COUNTIF('Cook log'!C2:C1000,A119)</f>
+        <v/>
+      </c>
+      <c r="F119" t="n">
+        <v>21</v>
+      </c>
+      <c r="G119">
+        <f>IF(C119="","Never cooked",IF(D119&lt;F119,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Oven baked chicken leg</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="C120">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A120)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A120)),"")</f>
+        <v/>
+      </c>
+      <c r="D120">
+        <f>IF(C120="","",TODAY()-C120)</f>
+        <v/>
+      </c>
+      <c r="E120">
+        <f>COUNTIF('Cook log'!C2:C1000,A120)</f>
+        <v/>
+      </c>
+      <c r="F120" t="n">
+        <v>21</v>
+      </c>
+      <c r="G120">
+        <f>IF(C120="","Never cooked",IF(D120&lt;F120,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Baked potatoes</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C121">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A121)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A121)),"")</f>
+        <v/>
+      </c>
+      <c r="D121">
+        <f>IF(C121="","",TODAY()-C121)</f>
+        <v/>
+      </c>
+      <c r="E121">
+        <f>COUNTIF('Cook log'!C2:C1000,A121)</f>
+        <v/>
+      </c>
+      <c r="F121" t="n">
+        <v>21</v>
+      </c>
+      <c r="G121">
+        <f>IF(C121="","Never cooked",IF(D121&lt;F121,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Aligot</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C122">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A122)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A122)),"")</f>
+        <v/>
+      </c>
+      <c r="D122">
+        <f>IF(C122="","",TODAY()-C122)</f>
+        <v/>
+      </c>
+      <c r="E122">
+        <f>COUNTIF('Cook log'!C2:C1000,A122)</f>
+        <v/>
+      </c>
+      <c r="F122" t="n">
+        <v>21</v>
+      </c>
+      <c r="G122">
+        <f>IF(C122="","Never cooked",IF(D122&lt;F122,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Baked pork chops</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="C123">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A123)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A123)),"")</f>
+        <v/>
+      </c>
+      <c r="D123">
+        <f>IF(C123="","",TODAY()-C123)</f>
+        <v/>
+      </c>
+      <c r="E123">
+        <f>COUNTIF('Cook log'!C2:C1000,A123)</f>
+        <v/>
+      </c>
+      <c r="F123" t="n">
+        <v>21</v>
+      </c>
+      <c r="G123">
+        <f>IF(C123="","Never cooked",IF(D123&lt;F123,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Japanese curry rice</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C124">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A124)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A124)),"")</f>
+        <v/>
+      </c>
+      <c r="D124">
+        <f>IF(C124="","",TODAY()-C124)</f>
+        <v/>
+      </c>
+      <c r="E124">
+        <f>COUNTIF('Cook log'!C2:C1000,A124)</f>
+        <v/>
+      </c>
+      <c r="F124" t="n">
+        <v>21</v>
+      </c>
+      <c r="G124">
+        <f>IF(C124="","Never cooked",IF(D124&lt;F124,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Campbell's mushroom soup</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C125">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A125)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A125)),"")</f>
+        <v/>
+      </c>
+      <c r="D125">
+        <f>IF(C125="","",TODAY()-C125)</f>
+        <v/>
+      </c>
+      <c r="E125">
+        <f>COUNTIF('Cook log'!C2:C1000,A125)</f>
+        <v/>
+      </c>
+      <c r="F125" t="n">
+        <v>21</v>
+      </c>
+      <c r="G125">
+        <f>IF(C125="","Never cooked",IF(D125&lt;F125,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Grilled asparagus</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C126">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A126)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A126)),"")</f>
+        <v/>
+      </c>
+      <c r="D126">
+        <f>IF(C126="","",TODAY()-C126)</f>
+        <v/>
+      </c>
+      <c r="E126">
+        <f>COUNTIF('Cook log'!C2:C1000,A126)</f>
+        <v/>
+      </c>
+      <c r="F126" t="n">
+        <v>21</v>
+      </c>
+      <c r="G126">
+        <f>IF(C126="","Never cooked",IF(D126&lt;F126,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Grilled broccoli &amp; carrots</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C127">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A127)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A127)),"")</f>
+        <v/>
+      </c>
+      <c r="D127">
+        <f>IF(C127="","",TODAY()-C127)</f>
+        <v/>
+      </c>
+      <c r="E127">
+        <f>COUNTIF('Cook log'!C2:C1000,A127)</f>
+        <v/>
+      </c>
+      <c r="F127" t="n">
+        <v>21</v>
+      </c>
+      <c r="G127">
+        <f>IF(C127="","Never cooked",IF(D127&lt;F127,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Crispy roast potatoes</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C128">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A128)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A128)),"")</f>
+        <v/>
+      </c>
+      <c r="D128">
+        <f>IF(C128="","",TODAY()-C128)</f>
+        <v/>
+      </c>
+      <c r="E128">
+        <f>COUNTIF('Cook log'!C2:C1000,A128)</f>
+        <v/>
+      </c>
+      <c r="F128" t="n">
+        <v>21</v>
+      </c>
+      <c r="G128">
+        <f>IF(C128="","Never cooked",IF(D128&lt;F128,"Cooldown","Due"))</f>
         <v/>
       </c>
     </row>

</xml_diff>